<commit_message>
Standardize CPI+ return targets by risk category, not by fund
DNA and Monarch models in the same risk category now share identical
CPI+ targets and nominal returns. DNA's targets are the house standard;
Monarch's are overridden to match (previously each Monarch model used
its own fund-of-funds' stated CPI+ band, or an extrapolated figure for
Income/Equity, which caused the two ranges to diverge — most visibly
at the Aggressive end, where Monarch showed 13.0% vs DNA's 11.5%).

Monarch's single Aggressive model uses DNA Aggressive Equity's 6.5%
target rather than Global Aggressive's 7.0%, since Monarch has only one
Aggressive model and it's SA/global-blended like Aggressive Equity.

Re-synced from the spreadsheet after applying the standardization there.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/DNA_Model_Portfolio_Metrics_130726.xlsx
+++ b/data/DNA_Model_Portfolio_Metrics_130726.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://omegacloudmail1-my.sharepoint.com/personal/marc_thomas_attooh_co_za/Documents/Desktop/DNA Invest/Blended Portfolio metrics/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2042" documentId="8_{258D6752-AA29-4249-BB06-E7A495CA3FAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6C8B8991-367F-4A27-880C-F2A7DAC293AD}"/>
+  <xr:revisionPtr revIDLastSave="2051" documentId="8_{258D6752-AA29-4249-BB06-E7A495CA3FAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7C72CF4C-3AB3-483C-86E4-2DE7CA66392A}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15210" yWindow="9480" windowWidth="7500" windowHeight="6000" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Portfolio Insights" sheetId="3" r:id="rId1"/>
@@ -596,15 +596,6 @@
     <t>Monarch Integrate Equity Portfolio</t>
   </si>
   <si>
-    <t>Return target basis:</t>
-  </si>
-  <si>
-    <t>- Mod Con / Moderate / Mod Aggressive: CPI+ target explicitly stated on the fact sheet (band shown; value used = midpoint). Rolling period differs by model: Mod Con 3yr, Moderate 5yr, Mod Aggressive 7yr.</t>
-  </si>
-  <si>
-    <t>- Income and Equity: NOT CPI+ mandated on the fact sheet (Income targets the ASISA Income sector average over rolling 2yr; Equity targets capital growth vs the ASISA EQ General sector). The CPI+1% and CPI+8% figures used here are EXTRAPOLATED from the 2%-per-notch pattern in the three stated targets (ModCon mid 2%, Moderate mid 4%, ModAgg mid 6%) - not disclosed by Monarch. Treat as an estimate only.</t>
-  </si>
-  <si>
     <t>Income</t>
   </si>
   <si>
@@ -702,6 +693,15 @@
   </si>
   <si>
     <t>7. Total Effective Cost for Mod Con / Moderate / Mod Aggressive = the TIC of the actual retail Cogence Discovery Dynamic Asset Optimiser Fund of Funds each Monarch model replicates (per each portfolio's stated objective; holdings match exactly). CONFIRMED via each fund's own MDD (30 Jun 2026): Cautious DAO FoF (Mod Con) TER 1.73%/TC 0.07%/TIC 1.80%; Moderate DAO FoF (Moderate) TER 1.83%/TC 0.13%/TIC 1.96%; Balanced DAO FoF (Mod Aggressive) TER 1.96%/TC 0.19%/TIC 2.15%. Corrected 2026-07-23: figures step up with risk (1.80/1.96/2.15%), NOT uniform - an earlier uniform 2.15% entry for all three was incorrect for Mod Con and Moderate and has been replaced with the verified per-model figures.</t>
+  </si>
+  <si>
+    <t>Return target basis (STANDARDIZED 2026-07-24):</t>
+  </si>
+  <si>
+    <t>CPI+ Return Target is now driven by RISK CATEGORY, not by each range's own funds - the DNA range's CPI+ targets are the house standard and are mirrored onto the matching Monarch risk category, so a DNA model and a Monarch model in the same risk category always show the same return target and (at a given inflation assumption) the same nominal expected return in the simulator.</t>
+  </si>
+  <si>
+    <t>Mapping: Conservative 1.0% | Moderately Conservative 2.5% | Moderate 3.5% | Moderately Aggressive 5.0% | Aggressive 6.5% (= DNA Aggressive Equity; DNA's other Aggressive model, Global Aggressive, targets 7.0% but Monarch has only one Aggressive model so Aggressive Equity was used - see chat decision 2026-07-24). This SUPERSEDES the fund-of-funds' own stated CPI+ bands (Mod Con 1-3%, Moderate 3-5%, Mod Aggressive 5-7%) and the earlier extrapolated Income/Equity figures used before 2026-07-24.</t>
   </si>
 </sst>
 </file>
@@ -712,7 +712,7 @@
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="&quot;CPI+&quot;0.0%"/>
   </numFmts>
-  <fonts count="38" x14ac:knownFonts="1">
+  <fonts count="37" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -932,12 +932,6 @@
       <sz val="10"/>
       <color rgb="FF0000FF"/>
       <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FFFF6600"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -1213,7 +1207,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="106">
+  <cellXfs count="105">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -1372,7 +1366,7 @@
     <xf numFmtId="0" fontId="27" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="164" fontId="23" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1381,13 +1375,10 @@
     <xf numFmtId="10" fontId="29" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="10" fontId="37" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="10" fontId="34" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="36" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="10" fontId="29" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1396,28 +1387,28 @@
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1441,7 +1432,7 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="10" fontId="37" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="29" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -5873,57 +5864,57 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A1" s="80" t="s">
+      <c r="A1" s="86" t="s">
         <v>35</v>
       </c>
-      <c r="B1" s="81"/>
-      <c r="C1" s="81"/>
-      <c r="D1" s="81"/>
-      <c r="E1" s="81"/>
-      <c r="F1" s="81"/>
-      <c r="G1" s="81"/>
-      <c r="H1" s="81"/>
-      <c r="I1" s="81"/>
-      <c r="J1" s="81"/>
-      <c r="K1" s="81"/>
-      <c r="L1" s="81"/>
-      <c r="M1" s="81"/>
-      <c r="N1" s="81"/>
+      <c r="B1" s="80"/>
+      <c r="C1" s="80"/>
+      <c r="D1" s="80"/>
+      <c r="E1" s="80"/>
+      <c r="F1" s="80"/>
+      <c r="G1" s="80"/>
+      <c r="H1" s="80"/>
+      <c r="I1" s="80"/>
+      <c r="J1" s="80"/>
+      <c r="K1" s="80"/>
+      <c r="L1" s="80"/>
+      <c r="M1" s="80"/>
+      <c r="N1" s="80"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="82" t="s">
+      <c r="A2" s="87" t="s">
         <v>158</v>
       </c>
-      <c r="B2" s="81"/>
-      <c r="C2" s="81"/>
-      <c r="D2" s="81"/>
-      <c r="E2" s="81"/>
-      <c r="F2" s="81"/>
-      <c r="G2" s="81"/>
-      <c r="H2" s="81"/>
-      <c r="I2" s="81"/>
-      <c r="J2" s="81"/>
-      <c r="K2" s="81"/>
-      <c r="L2" s="81"/>
-      <c r="M2" s="81"/>
-      <c r="N2" s="81"/>
+      <c r="B2" s="80"/>
+      <c r="C2" s="80"/>
+      <c r="D2" s="80"/>
+      <c r="E2" s="80"/>
+      <c r="F2" s="80"/>
+      <c r="G2" s="80"/>
+      <c r="H2" s="80"/>
+      <c r="I2" s="80"/>
+      <c r="J2" s="80"/>
+      <c r="K2" s="80"/>
+      <c r="L2" s="80"/>
+      <c r="M2" s="80"/>
+      <c r="N2" s="80"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="83" t="s">
         <v>36</v>
       </c>
-      <c r="B4" s="84"/>
-      <c r="C4" s="84"/>
+      <c r="B4" s="82"/>
+      <c r="C4" s="82"/>
       <c r="D4" s="83" t="s">
         <v>37</v>
       </c>
-      <c r="E4" s="84"/>
-      <c r="F4" s="84"/>
+      <c r="E4" s="82"/>
+      <c r="F4" s="82"/>
       <c r="G4" s="83" t="s">
         <v>39</v>
       </c>
-      <c r="H4" s="84"/>
-      <c r="I4" s="84"/>
+      <c r="H4" s="82"/>
+      <c r="I4" s="82"/>
       <c r="J4" s="83" t="s">
         <v>41</v>
       </c>
@@ -5931,120 +5922,120 @@
       <c r="L4" s="83"/>
     </row>
     <row r="5" spans="1:14" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A5" s="85">
+      <c r="A5" s="88">
         <f>COUNTA('Model Portfolios'!B8:B13)</f>
         <v>6</v>
       </c>
-      <c r="B5" s="84"/>
-      <c r="C5" s="84"/>
-      <c r="D5" s="87">
+      <c r="B5" s="82"/>
+      <c r="C5" s="82"/>
+      <c r="D5" s="89">
         <f>AVERAGE('Model Portfolios'!Q8:Q13)</f>
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="E5" s="84"/>
-      <c r="F5" s="84"/>
-      <c r="G5" s="88">
+      <c r="E5" s="82"/>
+      <c r="F5" s="82"/>
+      <c r="G5" s="84">
         <f>MAX('Model Portfolios'!R8:R13)-MIN('Model Portfolios'!R8:R13)</f>
         <v>6.0000000000000005E-2</v>
       </c>
-      <c r="H5" s="84"/>
-      <c r="I5" s="84"/>
-      <c r="J5" s="88">
+      <c r="H5" s="82"/>
+      <c r="I5" s="82"/>
+      <c r="J5" s="84">
         <f>MAX('Model Portfolios'!S8:S13)-MIN('Model Portfolios'!S8:S13)</f>
         <v>0.1051</v>
       </c>
-      <c r="K5" s="84"/>
-      <c r="L5" s="84"/>
+      <c r="K5" s="82"/>
+      <c r="L5" s="82"/>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A6" s="86" t="s">
+      <c r="A6" s="81" t="s">
         <v>157</v>
       </c>
-      <c r="B6" s="84"/>
-      <c r="C6" s="84"/>
-      <c r="D6" s="86" t="s">
+      <c r="B6" s="82"/>
+      <c r="C6" s="82"/>
+      <c r="D6" s="81" t="s">
         <v>38</v>
       </c>
-      <c r="E6" s="84"/>
-      <c r="F6" s="84"/>
-      <c r="G6" s="86" t="s">
+      <c r="E6" s="82"/>
+      <c r="F6" s="82"/>
+      <c r="G6" s="81" t="s">
         <v>40</v>
       </c>
-      <c r="H6" s="84"/>
-      <c r="I6" s="84"/>
-      <c r="J6" s="86" t="s">
+      <c r="H6" s="82"/>
+      <c r="I6" s="82"/>
+      <c r="J6" s="81" t="s">
         <v>171</v>
       </c>
-      <c r="K6" s="86"/>
-      <c r="L6" s="86"/>
+      <c r="K6" s="81"/>
+      <c r="L6" s="81"/>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A8" s="89" t="s">
+      <c r="A8" s="79" t="s">
         <v>42</v>
       </c>
-      <c r="B8" s="81"/>
-      <c r="C8" s="81"/>
-      <c r="D8" s="81"/>
-      <c r="E8" s="81"/>
-      <c r="F8" s="81"/>
-      <c r="G8" s="81"/>
-      <c r="H8" s="81"/>
-      <c r="I8" s="81"/>
-      <c r="J8" s="81"/>
-      <c r="K8" s="81"/>
-      <c r="L8" s="81"/>
-      <c r="M8" s="81"/>
-      <c r="N8" s="81"/>
+      <c r="B8" s="80"/>
+      <c r="C8" s="80"/>
+      <c r="D8" s="80"/>
+      <c r="E8" s="80"/>
+      <c r="F8" s="80"/>
+      <c r="G8" s="80"/>
+      <c r="H8" s="80"/>
+      <c r="I8" s="80"/>
+      <c r="J8" s="80"/>
+      <c r="K8" s="80"/>
+      <c r="L8" s="80"/>
+      <c r="M8" s="80"/>
+      <c r="N8" s="80"/>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A9" s="90" t="s">
+      <c r="A9" s="85" t="s">
         <v>172</v>
       </c>
-      <c r="B9" s="81"/>
-      <c r="C9" s="81"/>
-      <c r="D9" s="81"/>
-      <c r="E9" s="81"/>
-      <c r="F9" s="81"/>
-      <c r="G9" s="81"/>
-      <c r="H9" s="81"/>
-      <c r="I9" s="81"/>
-      <c r="J9" s="81"/>
-      <c r="K9" s="81"/>
-      <c r="L9" s="81"/>
-      <c r="M9" s="81"/>
-      <c r="N9" s="81"/>
+      <c r="B9" s="80"/>
+      <c r="C9" s="80"/>
+      <c r="D9" s="80"/>
+      <c r="E9" s="80"/>
+      <c r="F9" s="80"/>
+      <c r="G9" s="80"/>
+      <c r="H9" s="80"/>
+      <c r="I9" s="80"/>
+      <c r="J9" s="80"/>
+      <c r="K9" s="80"/>
+      <c r="L9" s="80"/>
+      <c r="M9" s="80"/>
+      <c r="N9" s="80"/>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A10" s="81"/>
-      <c r="B10" s="81"/>
-      <c r="C10" s="81"/>
-      <c r="D10" s="81"/>
-      <c r="E10" s="81"/>
-      <c r="F10" s="81"/>
-      <c r="G10" s="81"/>
-      <c r="H10" s="81"/>
-      <c r="I10" s="81"/>
-      <c r="J10" s="81"/>
-      <c r="K10" s="81"/>
-      <c r="L10" s="81"/>
-      <c r="M10" s="81"/>
-      <c r="N10" s="81"/>
+      <c r="A10" s="80"/>
+      <c r="B10" s="80"/>
+      <c r="C10" s="80"/>
+      <c r="D10" s="80"/>
+      <c r="E10" s="80"/>
+      <c r="F10" s="80"/>
+      <c r="G10" s="80"/>
+      <c r="H10" s="80"/>
+      <c r="I10" s="80"/>
+      <c r="J10" s="80"/>
+      <c r="K10" s="80"/>
+      <c r="L10" s="80"/>
+      <c r="M10" s="80"/>
+      <c r="N10" s="80"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" s="81"/>
-      <c r="B11" s="81"/>
-      <c r="C11" s="81"/>
-      <c r="D11" s="81"/>
-      <c r="E11" s="81"/>
-      <c r="F11" s="81"/>
-      <c r="G11" s="81"/>
-      <c r="H11" s="81"/>
-      <c r="I11" s="81"/>
-      <c r="J11" s="81"/>
-      <c r="K11" s="81"/>
-      <c r="L11" s="81"/>
-      <c r="M11" s="81"/>
-      <c r="N11" s="81"/>
+      <c r="A11" s="80"/>
+      <c r="B11" s="80"/>
+      <c r="C11" s="80"/>
+      <c r="D11" s="80"/>
+      <c r="E11" s="80"/>
+      <c r="F11" s="80"/>
+      <c r="G11" s="80"/>
+      <c r="H11" s="80"/>
+      <c r="I11" s="80"/>
+      <c r="J11" s="80"/>
+      <c r="K11" s="80"/>
+      <c r="L11" s="80"/>
+      <c r="M11" s="80"/>
+      <c r="N11" s="80"/>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
@@ -6704,15 +6695,15 @@
       </c>
     </row>
     <row r="50" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H50" s="89" t="s">
+      <c r="H50" s="79" t="s">
         <v>53</v>
       </c>
-      <c r="I50" s="81"/>
-      <c r="J50" s="81"/>
-      <c r="K50" s="81"/>
-      <c r="L50" s="81"/>
-      <c r="M50" s="81"/>
-      <c r="N50" s="81"/>
+      <c r="I50" s="80"/>
+      <c r="J50" s="80"/>
+      <c r="K50" s="80"/>
+      <c r="L50" s="80"/>
+      <c r="M50" s="80"/>
+      <c r="N50" s="80"/>
     </row>
     <row r="51" spans="8:14" ht="60" x14ac:dyDescent="0.25">
       <c r="H51" s="9">
@@ -6771,13 +6762,6 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="H50:N50"/>
-    <mergeCell ref="G6:I6"/>
-    <mergeCell ref="J4:L4"/>
-    <mergeCell ref="J5:L5"/>
-    <mergeCell ref="J6:L6"/>
-    <mergeCell ref="A8:N8"/>
-    <mergeCell ref="A9:N11"/>
     <mergeCell ref="A1:N1"/>
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A4:C4"/>
@@ -6788,6 +6772,13 @@
     <mergeCell ref="D6:F6"/>
     <mergeCell ref="G4:I4"/>
     <mergeCell ref="G5:I5"/>
+    <mergeCell ref="H50:N50"/>
+    <mergeCell ref="G6:I6"/>
+    <mergeCell ref="J4:L4"/>
+    <mergeCell ref="J5:L5"/>
+    <mergeCell ref="J6:L6"/>
+    <mergeCell ref="A8:N8"/>
+    <mergeCell ref="A9:N11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6810,48 +6801,48 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:20" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="B2" s="93" t="s">
+      <c r="B2" s="92" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="94"/>
-      <c r="D2" s="94"/>
-      <c r="E2" s="94"/>
-      <c r="F2" s="94"/>
-      <c r="G2" s="94"/>
-      <c r="H2" s="94"/>
-      <c r="I2" s="94"/>
-      <c r="J2" s="94"/>
-      <c r="K2" s="94"/>
-      <c r="L2" s="94"/>
-      <c r="M2" s="94"/>
-      <c r="N2" s="94"/>
-      <c r="O2" s="94"/>
-      <c r="P2" s="94"/>
-      <c r="Q2" s="94"/>
-      <c r="R2" s="94"/>
-      <c r="S2" s="94"/>
+      <c r="C2" s="93"/>
+      <c r="D2" s="93"/>
+      <c r="E2" s="93"/>
+      <c r="F2" s="93"/>
+      <c r="G2" s="93"/>
+      <c r="H2" s="93"/>
+      <c r="I2" s="93"/>
+      <c r="J2" s="93"/>
+      <c r="K2" s="93"/>
+      <c r="L2" s="93"/>
+      <c r="M2" s="93"/>
+      <c r="N2" s="93"/>
+      <c r="O2" s="93"/>
+      <c r="P2" s="93"/>
+      <c r="Q2" s="93"/>
+      <c r="R2" s="93"/>
+      <c r="S2" s="93"/>
     </row>
     <row r="3" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B3" s="95" t="s">
+      <c r="B3" s="94" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="96"/>
-      <c r="D3" s="96"/>
-      <c r="E3" s="96"/>
-      <c r="F3" s="96"/>
-      <c r="G3" s="96"/>
-      <c r="H3" s="96"/>
-      <c r="I3" s="96"/>
-      <c r="J3" s="96"/>
-      <c r="K3" s="96"/>
-      <c r="L3" s="96"/>
-      <c r="M3" s="96"/>
-      <c r="N3" s="96"/>
-      <c r="O3" s="96"/>
-      <c r="P3" s="96"/>
-      <c r="Q3" s="96"/>
-      <c r="R3" s="96"/>
-      <c r="S3" s="96"/>
+      <c r="C3" s="95"/>
+      <c r="D3" s="95"/>
+      <c r="E3" s="95"/>
+      <c r="F3" s="95"/>
+      <c r="G3" s="95"/>
+      <c r="H3" s="95"/>
+      <c r="I3" s="95"/>
+      <c r="J3" s="95"/>
+      <c r="K3" s="95"/>
+      <c r="L3" s="95"/>
+      <c r="M3" s="95"/>
+      <c r="N3" s="95"/>
+      <c r="O3" s="95"/>
+      <c r="P3" s="95"/>
+      <c r="Q3" s="95"/>
+      <c r="R3" s="95"/>
+      <c r="S3" s="95"/>
     </row>
     <row r="5" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B5" s="21" t="s">
@@ -7325,180 +7316,180 @@
       </c>
     </row>
     <row r="14" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B14" s="97" t="s">
+      <c r="B14" s="96" t="s">
         <v>59</v>
       </c>
-      <c r="C14" s="98"/>
-      <c r="D14" s="98"/>
-      <c r="E14" s="98"/>
-      <c r="F14" s="98"/>
-      <c r="G14" s="98"/>
-      <c r="H14" s="98"/>
-      <c r="I14" s="98"/>
-      <c r="J14" s="98"/>
-      <c r="K14" s="98"/>
-      <c r="L14" s="98"/>
-      <c r="M14" s="98"/>
-      <c r="N14" s="98"/>
-      <c r="O14" s="98"/>
-      <c r="P14" s="98"/>
-      <c r="Q14" s="98"/>
-      <c r="R14" s="98"/>
-      <c r="S14" s="98"/>
+      <c r="C14" s="97"/>
+      <c r="D14" s="97"/>
+      <c r="E14" s="97"/>
+      <c r="F14" s="97"/>
+      <c r="G14" s="97"/>
+      <c r="H14" s="97"/>
+      <c r="I14" s="97"/>
+      <c r="J14" s="97"/>
+      <c r="K14" s="97"/>
+      <c r="L14" s="97"/>
+      <c r="M14" s="97"/>
+      <c r="N14" s="97"/>
+      <c r="O14" s="97"/>
+      <c r="P14" s="97"/>
+      <c r="Q14" s="97"/>
+      <c r="R14" s="97"/>
+      <c r="S14" s="97"/>
     </row>
     <row r="16" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B16" s="99" t="s">
+      <c r="B16" s="98" t="s">
         <v>29</v>
       </c>
-      <c r="C16" s="100"/>
-      <c r="D16" s="100"/>
-      <c r="E16" s="100"/>
-      <c r="F16" s="100"/>
-      <c r="G16" s="100"/>
-      <c r="H16" s="100"/>
-      <c r="I16" s="100"/>
-      <c r="J16" s="100"/>
-      <c r="K16" s="100"/>
-      <c r="L16" s="100"/>
-      <c r="M16" s="100"/>
-      <c r="N16" s="100"/>
-      <c r="O16" s="100"/>
-      <c r="P16" s="100"/>
-      <c r="Q16" s="100"/>
-      <c r="R16" s="100"/>
-      <c r="S16" s="100"/>
+      <c r="C16" s="99"/>
+      <c r="D16" s="99"/>
+      <c r="E16" s="99"/>
+      <c r="F16" s="99"/>
+      <c r="G16" s="99"/>
+      <c r="H16" s="99"/>
+      <c r="I16" s="99"/>
+      <c r="J16" s="99"/>
+      <c r="K16" s="99"/>
+      <c r="L16" s="99"/>
+      <c r="M16" s="99"/>
+      <c r="N16" s="99"/>
+      <c r="O16" s="99"/>
+      <c r="P16" s="99"/>
+      <c r="Q16" s="99"/>
+      <c r="R16" s="99"/>
+      <c r="S16" s="99"/>
     </row>
     <row r="17" spans="2:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="101" t="s">
+      <c r="B17" s="100" t="s">
         <v>30</v>
       </c>
-      <c r="C17" s="102"/>
-      <c r="D17" s="102"/>
-      <c r="E17" s="102"/>
-      <c r="F17" s="102"/>
-      <c r="G17" s="102"/>
-      <c r="H17" s="102"/>
-      <c r="I17" s="102"/>
-      <c r="J17" s="102"/>
-      <c r="K17" s="102"/>
-      <c r="L17" s="102"/>
-      <c r="M17" s="102"/>
-      <c r="N17" s="102"/>
-      <c r="O17" s="102"/>
-      <c r="P17" s="102"/>
-      <c r="Q17" s="102"/>
-      <c r="R17" s="102"/>
-      <c r="S17" s="102"/>
+      <c r="C17" s="101"/>
+      <c r="D17" s="101"/>
+      <c r="E17" s="101"/>
+      <c r="F17" s="101"/>
+      <c r="G17" s="101"/>
+      <c r="H17" s="101"/>
+      <c r="I17" s="101"/>
+      <c r="J17" s="101"/>
+      <c r="K17" s="101"/>
+      <c r="L17" s="101"/>
+      <c r="M17" s="101"/>
+      <c r="N17" s="101"/>
+      <c r="O17" s="101"/>
+      <c r="P17" s="101"/>
+      <c r="Q17" s="101"/>
+      <c r="R17" s="101"/>
+      <c r="S17" s="101"/>
     </row>
     <row r="18" spans="2:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="103" t="s">
+      <c r="B18" s="102" t="s">
         <v>31</v>
       </c>
-      <c r="C18" s="104"/>
-      <c r="D18" s="104"/>
-      <c r="E18" s="104"/>
-      <c r="F18" s="104"/>
-      <c r="G18" s="104"/>
-      <c r="H18" s="104"/>
-      <c r="I18" s="104"/>
-      <c r="J18" s="104"/>
-      <c r="K18" s="104"/>
-      <c r="L18" s="104"/>
-      <c r="M18" s="104"/>
-      <c r="N18" s="104"/>
-      <c r="O18" s="104"/>
-      <c r="P18" s="104"/>
-      <c r="Q18" s="104"/>
-      <c r="R18" s="104"/>
-      <c r="S18" s="104"/>
+      <c r="C18" s="103"/>
+      <c r="D18" s="103"/>
+      <c r="E18" s="103"/>
+      <c r="F18" s="103"/>
+      <c r="G18" s="103"/>
+      <c r="H18" s="103"/>
+      <c r="I18" s="103"/>
+      <c r="J18" s="103"/>
+      <c r="K18" s="103"/>
+      <c r="L18" s="103"/>
+      <c r="M18" s="103"/>
+      <c r="N18" s="103"/>
+      <c r="O18" s="103"/>
+      <c r="P18" s="103"/>
+      <c r="Q18" s="103"/>
+      <c r="R18" s="103"/>
+      <c r="S18" s="103"/>
     </row>
     <row r="19" spans="2:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="103" t="s">
+      <c r="B19" s="102" t="s">
         <v>32</v>
       </c>
-      <c r="C19" s="104"/>
-      <c r="D19" s="104"/>
-      <c r="E19" s="104"/>
-      <c r="F19" s="104"/>
-      <c r="G19" s="104"/>
-      <c r="H19" s="104"/>
-      <c r="I19" s="104"/>
-      <c r="J19" s="104"/>
-      <c r="K19" s="104"/>
-      <c r="L19" s="104"/>
-      <c r="M19" s="104"/>
-      <c r="N19" s="104"/>
-      <c r="O19" s="104"/>
-      <c r="P19" s="104"/>
-      <c r="Q19" s="104"/>
-      <c r="R19" s="104"/>
-      <c r="S19" s="104"/>
+      <c r="C19" s="103"/>
+      <c r="D19" s="103"/>
+      <c r="E19" s="103"/>
+      <c r="F19" s="103"/>
+      <c r="G19" s="103"/>
+      <c r="H19" s="103"/>
+      <c r="I19" s="103"/>
+      <c r="J19" s="103"/>
+      <c r="K19" s="103"/>
+      <c r="L19" s="103"/>
+      <c r="M19" s="103"/>
+      <c r="N19" s="103"/>
+      <c r="O19" s="103"/>
+      <c r="P19" s="103"/>
+      <c r="Q19" s="103"/>
+      <c r="R19" s="103"/>
+      <c r="S19" s="103"/>
     </row>
     <row r="20" spans="2:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="103" t="s">
+      <c r="B20" s="102" t="s">
         <v>33</v>
       </c>
-      <c r="C20" s="104"/>
-      <c r="D20" s="104"/>
-      <c r="E20" s="104"/>
-      <c r="F20" s="104"/>
-      <c r="G20" s="104"/>
-      <c r="H20" s="104"/>
-      <c r="I20" s="104"/>
-      <c r="J20" s="104"/>
-      <c r="K20" s="104"/>
-      <c r="L20" s="104"/>
-      <c r="M20" s="104"/>
-      <c r="N20" s="104"/>
-      <c r="O20" s="104"/>
-      <c r="P20" s="104"/>
-      <c r="Q20" s="104"/>
-      <c r="R20" s="104"/>
-      <c r="S20" s="104"/>
+      <c r="C20" s="103"/>
+      <c r="D20" s="103"/>
+      <c r="E20" s="103"/>
+      <c r="F20" s="103"/>
+      <c r="G20" s="103"/>
+      <c r="H20" s="103"/>
+      <c r="I20" s="103"/>
+      <c r="J20" s="103"/>
+      <c r="K20" s="103"/>
+      <c r="L20" s="103"/>
+      <c r="M20" s="103"/>
+      <c r="N20" s="103"/>
+      <c r="O20" s="103"/>
+      <c r="P20" s="103"/>
+      <c r="Q20" s="103"/>
+      <c r="R20" s="103"/>
+      <c r="S20" s="103"/>
     </row>
     <row r="21" spans="2:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="103" t="s">
+      <c r="B21" s="102" t="s">
         <v>34</v>
       </c>
-      <c r="C21" s="104"/>
-      <c r="D21" s="104"/>
-      <c r="E21" s="104"/>
-      <c r="F21" s="104"/>
-      <c r="G21" s="104"/>
-      <c r="H21" s="104"/>
-      <c r="I21" s="104"/>
-      <c r="J21" s="104"/>
-      <c r="K21" s="104"/>
-      <c r="L21" s="104"/>
-      <c r="M21" s="104"/>
-      <c r="N21" s="104"/>
-      <c r="O21" s="104"/>
-      <c r="P21" s="104"/>
-      <c r="Q21" s="104"/>
-      <c r="R21" s="104"/>
-      <c r="S21" s="104"/>
+      <c r="C21" s="103"/>
+      <c r="D21" s="103"/>
+      <c r="E21" s="103"/>
+      <c r="F21" s="103"/>
+      <c r="G21" s="103"/>
+      <c r="H21" s="103"/>
+      <c r="I21" s="103"/>
+      <c r="J21" s="103"/>
+      <c r="K21" s="103"/>
+      <c r="L21" s="103"/>
+      <c r="M21" s="103"/>
+      <c r="N21" s="103"/>
+      <c r="O21" s="103"/>
+      <c r="P21" s="103"/>
+      <c r="Q21" s="103"/>
+      <c r="R21" s="103"/>
+      <c r="S21" s="103"/>
     </row>
     <row r="22" spans="2:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="91" t="s">
+      <c r="B22" s="90" t="s">
         <v>169</v>
       </c>
-      <c r="C22" s="92"/>
-      <c r="D22" s="92"/>
-      <c r="E22" s="92"/>
-      <c r="F22" s="92"/>
-      <c r="G22" s="92"/>
-      <c r="H22" s="92"/>
-      <c r="I22" s="92"/>
-      <c r="J22" s="92"/>
-      <c r="K22" s="92"/>
-      <c r="L22" s="92"/>
-      <c r="M22" s="92"/>
-      <c r="N22" s="92"/>
-      <c r="O22" s="92"/>
-      <c r="P22" s="92"/>
-      <c r="Q22" s="92"/>
-      <c r="R22" s="92"/>
-      <c r="S22" s="92"/>
+      <c r="C22" s="91"/>
+      <c r="D22" s="91"/>
+      <c r="E22" s="91"/>
+      <c r="F22" s="91"/>
+      <c r="G22" s="91"/>
+      <c r="H22" s="91"/>
+      <c r="I22" s="91"/>
+      <c r="J22" s="91"/>
+      <c r="K22" s="91"/>
+      <c r="L22" s="91"/>
+      <c r="M22" s="91"/>
+      <c r="N22" s="91"/>
+      <c r="O22" s="91"/>
+      <c r="P22" s="91"/>
+      <c r="Q22" s="91"/>
+      <c r="R22" s="91"/>
+      <c r="S22" s="91"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -7558,20 +7549,20 @@
       <c r="L1" s="39"/>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A2" s="79" t="s">
+      <c r="A2" s="78" t="s">
         <v>115</v>
       </c>
-      <c r="B2" s="79"/>
-      <c r="C2" s="79"/>
-      <c r="D2" s="79"/>
-      <c r="E2" s="79"/>
-      <c r="F2" s="79"/>
-      <c r="G2" s="79"/>
-      <c r="H2" s="79"/>
-      <c r="I2" s="79"/>
-      <c r="J2" s="79"/>
-      <c r="K2" s="79"/>
-      <c r="L2" s="79"/>
+      <c r="B2" s="78"/>
+      <c r="C2" s="78"/>
+      <c r="D2" s="78"/>
+      <c r="E2" s="78"/>
+      <c r="F2" s="78"/>
+      <c r="G2" s="78"/>
+      <c r="H2" s="78"/>
+      <c r="I2" s="78"/>
+      <c r="J2" s="78"/>
+      <c r="K2" s="78"/>
+      <c r="L2" s="78"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="39"/>
@@ -10003,26 +9994,26 @@
       <c r="R1" s="39"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A2" s="79" t="s">
-        <v>198</v>
-      </c>
-      <c r="B2" s="79"/>
-      <c r="C2" s="79"/>
-      <c r="D2" s="79"/>
-      <c r="E2" s="79"/>
-      <c r="F2" s="79"/>
-      <c r="G2" s="79"/>
-      <c r="H2" s="79"/>
-      <c r="I2" s="79"/>
-      <c r="J2" s="79"/>
-      <c r="K2" s="79"/>
-      <c r="L2" s="79"/>
-      <c r="M2" s="79"/>
-      <c r="N2" s="79"/>
-      <c r="O2" s="79"/>
-      <c r="P2" s="79"/>
-      <c r="Q2" s="79"/>
-      <c r="R2" s="79"/>
+      <c r="A2" s="78" t="s">
+        <v>195</v>
+      </c>
+      <c r="B2" s="78"/>
+      <c r="C2" s="78"/>
+      <c r="D2" s="78"/>
+      <c r="E2" s="78"/>
+      <c r="F2" s="78"/>
+      <c r="G2" s="78"/>
+      <c r="H2" s="78"/>
+      <c r="I2" s="78"/>
+      <c r="J2" s="78"/>
+      <c r="K2" s="78"/>
+      <c r="L2" s="78"/>
+      <c r="M2" s="78"/>
+      <c r="N2" s="78"/>
+      <c r="O2" s="78"/>
+      <c r="P2" s="78"/>
+      <c r="Q2" s="78"/>
+      <c r="R2" s="78"/>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" s="39"/>
@@ -10049,7 +10040,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="39" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="C4" s="39"/>
       <c r="D4" s="39" t="s">
@@ -10128,13 +10119,13 @@
         <v>16</v>
       </c>
       <c r="M6" s="43" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="N6" s="43" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="O6" s="43" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="P6" s="43" t="s">
         <v>18</v>
@@ -10193,14 +10184,14 @@
       <c r="O7" s="76">
         <v>1.4800000000000001E-2</v>
       </c>
-      <c r="P7" s="77">
+      <c r="P7" s="104">
         <v>0.01</v>
       </c>
       <c r="Q7" s="44">
         <v>3.9100000000000003E-2</v>
       </c>
       <c r="R7" s="39" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.25">
@@ -10247,17 +10238,17 @@
       <c r="N8" s="74">
         <v>1.2999999999999999E-2</v>
       </c>
-      <c r="O8" s="105">
+      <c r="O8" s="76">
         <v>1.7999999999999999E-2</v>
       </c>
-      <c r="P8" s="74">
-        <v>0.02</v>
+      <c r="P8" s="104">
+        <v>2.5000000000000001E-2</v>
       </c>
       <c r="Q8" s="48">
         <v>7.6300000000000007E-2</v>
       </c>
       <c r="R8" s="47" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.25">
@@ -10304,17 +10295,17 @@
       <c r="N9" s="52">
         <v>1.4E-2</v>
       </c>
-      <c r="O9" s="105">
+      <c r="O9" s="76">
         <v>1.9599999999999999E-2</v>
       </c>
-      <c r="P9" s="52">
-        <v>0.04</v>
+      <c r="P9" s="104">
+        <v>3.5000000000000003E-2</v>
       </c>
       <c r="Q9" s="44">
         <v>8.6599999999999996E-2</v>
       </c>
       <c r="R9" s="39" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.25">
@@ -10361,17 +10352,17 @@
       <c r="N10" s="74">
         <v>1.47E-2</v>
       </c>
-      <c r="O10" s="105">
+      <c r="O10" s="76">
         <v>2.1499999999999998E-2</v>
       </c>
-      <c r="P10" s="74">
-        <v>0.06</v>
+      <c r="P10" s="104">
+        <v>0.05</v>
       </c>
       <c r="Q10" s="48">
         <v>9.5899999999999999E-2</v>
       </c>
       <c r="R10" s="47" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.25">
@@ -10421,14 +10412,14 @@
       <c r="O11" s="76">
         <v>2.4899999999999999E-2</v>
       </c>
-      <c r="P11" s="77">
-        <v>0.08</v>
+      <c r="P11" s="104">
+        <v>6.5000000000000002E-2</v>
       </c>
       <c r="Q11" s="44">
         <v>0.10630000000000001</v>
       </c>
       <c r="R11" s="72" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.25">
@@ -10453,7 +10444,7 @@
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13" s="39" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="B13" s="39"/>
       <c r="C13" s="39"/>
@@ -10495,7 +10486,7 @@
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A15" s="75" t="s">
-        <v>186</v>
+        <v>219</v>
       </c>
       <c r="B15" s="39"/>
       <c r="C15" s="39"/>
@@ -10517,7 +10508,7 @@
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A16" s="75" t="s">
-        <v>187</v>
+        <v>220</v>
       </c>
       <c r="B16" s="39"/>
       <c r="C16" s="39"/>
@@ -10539,7 +10530,7 @@
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A17" s="75" t="s">
-        <v>188</v>
+        <v>221</v>
       </c>
       <c r="B17" s="39"/>
       <c r="C17" s="39"/>
@@ -10581,7 +10572,7 @@
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A19" s="75" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="B19" s="39"/>
       <c r="C19" s="39"/>
@@ -10623,7 +10614,7 @@
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A21" s="42" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="B21" s="39"/>
       <c r="C21" s="39"/>
@@ -10654,10 +10645,10 @@
         <v>107</v>
       </c>
       <c r="D22" s="43" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="E22" s="43" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="F22" s="39"/>
       <c r="G22" s="39"/>
@@ -10675,10 +10666,10 @@
     </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A23" s="39" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="B23" s="39" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="C23" s="45">
         <v>0.8</v>
@@ -10705,10 +10696,10 @@
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A24" s="47" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="B24" s="47" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="C24" s="53">
         <v>0.2</v>
@@ -10735,10 +10726,10 @@
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A25" s="39" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="B25" s="39" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="C25" s="45">
         <v>0.47099999999999997</v>
@@ -10765,10 +10756,10 @@
     </row>
     <row r="26" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A26" s="47" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="B26" s="47" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C26" s="53">
         <v>0.30499999999999999</v>
@@ -10795,10 +10786,10 @@
     </row>
     <row r="27" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A27" s="39" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="B27" s="39" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="C27" s="45">
         <v>8.7999999999999995E-2</v>
@@ -10825,10 +10816,10 @@
     </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A28" s="47" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="B28" s="47" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="C28" s="53">
         <v>7.1999999999999995E-2</v>
@@ -10855,10 +10846,10 @@
     </row>
     <row r="29" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A29" s="39" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="B29" s="39" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="C29" s="45">
         <v>4.8000000000000001E-2</v>
@@ -10885,10 +10876,10 @@
     </row>
     <row r="30" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A30" s="47" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="B30" s="47" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="C30" s="53">
         <v>8.0000000000000002E-3</v>
@@ -10913,10 +10904,10 @@
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A31" s="39" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="B31" s="39" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="C31" s="45">
         <v>5.0000000000000001E-3</v>
@@ -10943,10 +10934,10 @@
     </row>
     <row r="32" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A32" s="47" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="B32" s="47" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="C32" s="53">
         <v>3.0000000000000001E-3</v>
@@ -10974,12 +10965,12 @@
         <v>24</v>
       </c>
       <c r="B33" s="39" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C33" s="45">
         <v>0.35799999999999998</v>
       </c>
-      <c r="D33" s="78">
+      <c r="D33" s="77">
         <v>1.43E-2</v>
       </c>
       <c r="E33" s="44">
@@ -11004,7 +10995,7 @@
         <v>24</v>
       </c>
       <c r="B34" s="47" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="C34" s="53">
         <v>0.30299999999999999</v>
@@ -11034,7 +11025,7 @@
         <v>24</v>
       </c>
       <c r="B35" s="39" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="C35" s="45">
         <v>0.17</v>
@@ -11064,7 +11055,7 @@
         <v>24</v>
       </c>
       <c r="B36" s="47" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="C36" s="53">
         <v>0.115</v>
@@ -11094,7 +11085,7 @@
         <v>24</v>
       </c>
       <c r="B37" s="39" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="C37" s="45">
         <v>3.9E-2</v>
@@ -11124,7 +11115,7 @@
         <v>24</v>
       </c>
       <c r="B38" s="47" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="C38" s="53">
         <v>8.0000000000000002E-3</v>
@@ -11152,7 +11143,7 @@
         <v>24</v>
       </c>
       <c r="B39" s="39" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="C39" s="45">
         <v>5.0000000000000001E-3</v>
@@ -11182,7 +11173,7 @@
         <v>24</v>
       </c>
       <c r="B40" s="47" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="C40" s="53">
         <v>2E-3</v>
@@ -11207,15 +11198,15 @@
     </row>
     <row r="41" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A41" s="39" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="B41" s="39" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C41" s="45">
         <v>0.36899999999999999</v>
       </c>
-      <c r="D41" s="78">
+      <c r="D41" s="77">
         <v>1.43E-2</v>
       </c>
       <c r="E41" s="44">
@@ -11237,10 +11228,10 @@
     </row>
     <row r="42" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A42" s="47" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="B42" s="47" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="C42" s="53">
         <v>0.255</v>
@@ -11267,10 +11258,10 @@
     </row>
     <row r="43" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A43" s="39" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="B43" s="39" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="C43" s="45">
         <v>0.17699999999999999</v>
@@ -11297,10 +11288,10 @@
     </row>
     <row r="44" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A44" s="47" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="B44" s="47" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="C44" s="53">
         <v>0.17599999999999999</v>
@@ -11327,10 +11318,10 @@
     </row>
     <row r="45" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A45" s="39" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="B45" s="39" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="C45" s="45">
         <v>8.0000000000000002E-3</v>
@@ -11357,10 +11348,10 @@
     </row>
     <row r="46" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A46" s="47" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="B46" s="47" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="C46" s="53">
         <v>7.0000000000000001E-3</v>
@@ -11385,10 +11376,10 @@
     </row>
     <row r="47" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A47" s="39" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="B47" s="39" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="C47" s="45">
         <v>5.0000000000000001E-3</v>
@@ -11415,10 +11406,10 @@
     </row>
     <row r="48" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A48" s="47" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="B48" s="47" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="C48" s="53">
         <v>2E-3</v>
@@ -11443,10 +11434,10 @@
     </row>
     <row r="49" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A49" s="39" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="B49" s="39" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="C49" s="45">
         <v>0.85</v>
@@ -11473,10 +11464,10 @@
     </row>
     <row r="50" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A50" s="47" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="B50" s="47" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="C50" s="53">
         <v>0.15</v>
@@ -11545,7 +11536,7 @@
     </row>
     <row r="53" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A53" s="75" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="B53" s="39"/>
       <c r="C53" s="39"/>
@@ -11567,7 +11558,7 @@
     </row>
     <row r="54" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A54" s="75" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="B54" s="39"/>
       <c r="C54" s="39"/>
@@ -11589,7 +11580,7 @@
     </row>
     <row r="55" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A55" s="75" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="B55" s="39"/>
       <c r="C55" s="39"/>
@@ -11611,7 +11602,7 @@
     </row>
     <row r="56" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A56" s="75" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="B56" s="39"/>
       <c r="C56" s="39"/>
@@ -11633,7 +11624,7 @@
     </row>
     <row r="57" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A57" s="75" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="B57" s="39"/>
       <c r="C57" s="39"/>
@@ -11655,7 +11646,7 @@
     </row>
     <row r="58" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A58" s="75" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="B58" s="39"/>
       <c r="C58" s="39"/>
@@ -11677,7 +11668,7 @@
     </row>
     <row r="59" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A59" s="69" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
     </row>
   </sheetData>

</xml_diff>